<commit_message>
Add preference-only track assignment mode
</commit_message>
<xml_diff>
--- a/готовое_решение/тест/01_исходный_файл/выход/результат_распределения.xlsx
+++ b/готовое_решение/тест/01_исходный_файл/выход/результат_распределения.xlsx
@@ -3,9 +3,10 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
     <sheet name="Результат" sheetId="1" r:id="rId1"/>
-    <sheet name="Количество_по_трекам" sheetId="2" r:id="rId2"/>
-    <sheet name="Без_выбора" sheetId="3" r:id="rId3"/>
-    <sheet name="Приоритеты_1_2" sheetId="4" r:id="rId4"/>
+    <sheet name="Гипотеза" sheetId="2" r:id="rId2"/>
+    <sheet name="Количество_по_трекам" sheetId="3" r:id="rId3"/>
+    <sheet name="Без_выбора" sheetId="4" r:id="rId4"/>
+    <sheet name="Приоритеты_1_2" sheetId="5" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
@@ -73,15 +74,25 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>режим распределения</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>попадание по предпочтению</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>выбор трека</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>статус без выбора</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>приоритеты</t>
         </is>
@@ -106,10 +117,20 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>выбор указан</t>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>приоритет 1</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
         <is>
           <t>Трек А: 3, Трек В: 2, Трек С: 1</t>
         </is>
@@ -134,15 +155,25 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>выбор не указан</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>выбор не указан</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>статус не указан</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>Трек А: 0, Трек В: 0, Трек С: 0</t>
         </is>
@@ -167,10 +198,20 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>выбор указан</t>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>приоритет 1</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
         <is>
           <t>Трек А: 3, Трек В: 2, Трек С: 1</t>
         </is>
@@ -195,10 +236,20 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>выбор указан</t>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>приоритет 1</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
         <is>
           <t>Трек А: 1, Трек В: 3, Трек С: 2</t>
         </is>
@@ -223,15 +274,25 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>выбор не указан</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>выбор не указан</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>статус не указан</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>Трек А: 0, Трек В: 0, Трек С: 0</t>
         </is>
@@ -256,10 +317,20 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>выбор указан</t>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>приоритет 1</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
         <is>
           <t>Трек А: 3, Трек В: 2, Трек С: 1</t>
         </is>
@@ -284,10 +355,20 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>выбор указан</t>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>приоритет 1</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
         <is>
           <t>Трек А: 3, Трек В: 1, Трек С: 2</t>
         </is>
@@ -312,10 +393,20 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>выбор указан</t>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>приоритет 1</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
         <is>
           <t>Трек А: 3, Трек В: 1, Трек С: 2</t>
         </is>
@@ -340,15 +431,25 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
           <t>выбор не указан</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>выбор не указан</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
         <is>
           <t>статус не указан</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>Трек А: 0, Трек В: 0, Трек С: 0</t>
         </is>
@@ -373,10 +474,20 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>выбор указан</t>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>приоритет 1</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
         <is>
           <t>Трек А: 2, Трек В: 1, Трек С: 3</t>
         </is>
@@ -401,10 +512,20 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>выбор указан</t>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>приоритет 1</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
         <is>
           <t>Трек А: 3, Трек В: 2, Трек С: 1</t>
         </is>
@@ -429,10 +550,20 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>выбор указан</t>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>приоритет 1</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
         <is>
           <t>Трек А: 2, Трек В: 1, Трек С: 3</t>
         </is>
@@ -457,15 +588,25 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
           <t>выбор не указан</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>выбор не указан</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
         <is>
           <t>статус не указан</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>Трек А: 0, Трек В: 0, Трек С: 0</t>
         </is>
@@ -490,10 +631,20 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>выбор указан</t>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>приоритет 1</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
         <is>
           <t>Трек А: 1, Трек В: 3, Трек С: 2</t>
         </is>
@@ -518,10 +669,20 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>выбор указан</t>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>приоритет 1</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
         <is>
           <t>Трек А: 3, Трек В: 2, Трек С: 1</t>
         </is>
@@ -546,10 +707,20 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>выбор указан</t>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>приоритет 1</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
         <is>
           <t>Трек А: 3, Трек В: 1, Трек С: 2</t>
         </is>
@@ -574,15 +745,25 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
           <t>выбор не указан</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>выбор не указан</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
         <is>
           <t>статус не указан</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>Трек А: 0, Трек В: 0, Трек С: 0</t>
         </is>
@@ -607,10 +788,20 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>выбор указан</t>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>приоритет 1</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
         <is>
           <t>Трек А: 3, Трек В: 1, Трек С: 2</t>
         </is>
@@ -635,10 +826,20 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>выбор указан</t>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>приоритет 1</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
         <is>
           <t>Трек А: 3, Трек В: 2, Трек С: 1</t>
         </is>
@@ -663,10 +864,20 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>выбор указан</t>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>приоритет 1</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
         <is>
           <t>Трек А: 1, Трек В: 3, Трек С: 2</t>
         </is>
@@ -691,10 +902,20 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>выбор указан</t>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>приоритет 1</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
         <is>
           <t>Трек А: 1, Трек В: 2, Трек С: 3</t>
         </is>
@@ -719,15 +940,25 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
           <t>выбор не указан</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>выбор не указан</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
         <is>
           <t>статус не указан</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>Трек А: 0, Трек В: 0, Трек С: 0</t>
         </is>
@@ -752,10 +983,20 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>выбор указан</t>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>приоритет 1</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
         <is>
           <t>Трек А: 2, Трек В: 3, Трек С: 1</t>
         </is>
@@ -780,10 +1021,20 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>выбор указан</t>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>приоритет 1</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
         <is>
           <t>Трек А: 2, Трек В: 1, Трек С: 3</t>
         </is>
@@ -808,10 +1059,20 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>выбор указан</t>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>приоритет 1</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
         <is>
           <t>Трек А: 2, Трек В: 1, Трек С: 3</t>
         </is>
@@ -836,10 +1097,20 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>выбор указан</t>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>приоритет 1</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
         <is>
           <t>Трек А: 2, Трек В: 3, Трек С: 1</t>
         </is>
@@ -864,10 +1135,20 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>выбор указан</t>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>приоритет 1</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
         <is>
           <t>Трек А: 1, Трек В: 2, Трек С: 3</t>
         </is>
@@ -892,10 +1173,20 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>выбор указан</t>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>приоритет 1</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
         <is>
           <t>Трек А: 2, Трек В: 3, Трек С: 1</t>
         </is>
@@ -920,10 +1211,20 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>выбор указан</t>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>приоритет 1</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
         <is>
           <t>Трек А: 3, Трек В: 2, Трек С: 1</t>
         </is>
@@ -948,10 +1249,20 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>выбор указан</t>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>приоритет 1</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
         <is>
           <t>Трек А: 3, Трек В: 2, Трек С: 1</t>
         </is>
@@ -976,10 +1287,20 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>выбор указан</t>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>приоритет 1</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
         <is>
           <t>Трек А: 3, Трек В: 1, Трек С: 2</t>
         </is>
@@ -1004,10 +1325,20 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>выбор указан</t>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>приоритет 1</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
         <is>
           <t>Трек А: 1, Трек В: 2, Трек С: 3</t>
         </is>
@@ -1032,10 +1363,20 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>выбор указан</t>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>приоритет 1</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
         <is>
           <t>Трек А: 2, Трек В: 1, Трек С: 3</t>
         </is>
@@ -1060,15 +1401,25 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
           <t>выбор не указан</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>выбор не указан</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
         <is>
           <t>статус не указан</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="I35" t="inlineStr">
         <is>
           <t>Трек А: 0, Трек В: 0, Трек С: 0</t>
         </is>
@@ -1093,10 +1444,20 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>выбор указан</t>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>приоритет 1</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
         <is>
           <t>Трек А: 1, Трек В: 2, Трек С: 3</t>
         </is>
@@ -1121,10 +1482,20 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>выбор указан</t>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>приоритет 1</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
         <is>
           <t>Трек А: 3, Трек В: 2, Трек С: 1</t>
         </is>
@@ -1149,15 +1520,25 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
           <t>выбор не указан</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>выбор не указан</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
         <is>
           <t>статус не указан</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
+      <c r="I38" t="inlineStr">
         <is>
           <t>Трек А: 0, Трек В: 0, Трек С: 0</t>
         </is>
@@ -1182,10 +1563,20 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>выбор указан</t>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>приоритет 1</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
         <is>
           <t>Трек А: 1, Трек В: 3, Трек С: 2</t>
         </is>
@@ -1210,15 +1601,25 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
           <t>выбор не указан</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>выбор не указан</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
         <is>
           <t>статус не указан</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
+      <c r="I40" t="inlineStr">
         <is>
           <t>Трек А: 0, Трек В: 0, Трек С: 0</t>
         </is>
@@ -1243,10 +1644,20 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>выбор указан</t>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>приоритет 1</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
         <is>
           <t>Трек А: 2, Трек В: 3, Трек С: 1</t>
         </is>
@@ -1271,15 +1682,25 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
           <t>выбор не указан</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>выбор не указан</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
         <is>
           <t>статус не указан</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
+      <c r="I42" t="inlineStr">
         <is>
           <t>Трек А: 0, Трек В: 0, Трек С: 0</t>
         </is>
@@ -1304,10 +1725,20 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>выбор указан</t>
+          <t>с рейтингом</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>приоритет 1</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
+        <is>
+          <t>выбор указан</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
         <is>
           <t>Трек А: 3, Трек В: 1, Трек С: 2</t>
         </is>
@@ -1323,71 +1754,129 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>трек</t>
+          <t>параметр</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>назначено студентов</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>приоритет 1</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>приоритет 1 или 2</t>
+          <t>значение</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Трек А</t>
-        </is>
-      </c>
-      <c r="B2">
-        <v>14</v>
-      </c>
-      <c r="C2">
-        <v>8</v>
-      </c>
-      <c r="D2">
-        <v>17</v>
+          <t>режим распределения</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>с учетом рейтинга</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Трек В</t>
-        </is>
-      </c>
-      <c r="B3">
-        <v>14</v>
-      </c>
-      <c r="C3">
-        <v>11</v>
-      </c>
-      <c r="D3">
-        <v>24</v>
+          <t>оценки участвуют в распределении</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Трек С</t>
+          <t>всего студентов</t>
         </is>
       </c>
       <c r="B4">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>студентов с указанными предпочтениями</t>
+        </is>
+      </c>
+      <c r="B5">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>студентов без выбора</t>
+        </is>
+      </c>
+      <c r="B6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>назначено на приоритет 1</t>
+        </is>
+      </c>
+      <c r="B7">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>назначено на приоритет 2</t>
+        </is>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>назначено вне приоритетов или без выбора</t>
+        </is>
+      </c>
+      <c r="B9">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>минимум по треку</t>
+        </is>
+      </c>
+      <c r="B10">
         <v>14</v>
       </c>
-      <c r="C4">
-        <v>13</v>
-      </c>
-      <c r="D4">
-        <v>23</v>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>максимум по треку</t>
+        </is>
+      </c>
+      <c r="B11">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>гипотеза</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>используется режим с рейтингом</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1400,258 +1889,71 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>id ученика</t>
+          <t>трек</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>трек</t>
+          <t>назначено студентов</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>место в рейтинге</t>
+          <t>приоритет 1</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>рейтинг</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>статус без выбора</t>
+          <t>приоритет 1 или 2</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>637756</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
           <t>Трек А</t>
         </is>
       </c>
+      <c r="B2">
+        <v>14</v>
+      </c>
       <c r="C2">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D2">
-        <v>100.004709</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>статус не указан</t>
-        </is>
+        <v>17</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>366609</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
           <t>Трек В</t>
         </is>
       </c>
+      <c r="B3">
+        <v>14</v>
+      </c>
       <c r="C3">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="D3">
-        <v>100.004692</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>статус не указан</t>
-        </is>
+        <v>24</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>449867</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Трек А</t>
-        </is>
+          <t>Трек С</t>
+        </is>
+      </c>
+      <c r="B4">
+        <v>14</v>
       </c>
       <c r="C4">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D4">
-        <v>99.492375</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>статус не указан</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>302756</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Трек А</t>
-        </is>
-      </c>
-      <c r="C5">
-        <v>13</v>
-      </c>
-      <c r="D5">
-        <v>97.987142</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>статус не указан</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>254592</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Трек А</t>
-        </is>
-      </c>
-      <c r="C6">
-        <v>17</v>
-      </c>
-      <c r="D6">
-        <v>96.805618</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>статус не указан</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>473699</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Трек С</t>
-        </is>
-      </c>
-      <c r="C7">
-        <v>22</v>
-      </c>
-      <c r="D7">
-        <v>95.028425</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>статус не указан</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>406855</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Трек А</t>
-        </is>
-      </c>
-      <c r="C8">
-        <v>34</v>
-      </c>
-      <c r="D8">
-        <v>87.061286</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>статус не указан</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>754466</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Трек В</t>
-        </is>
-      </c>
-      <c r="C9">
-        <v>37</v>
-      </c>
-      <c r="D9">
-        <v>83.014029</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>статус не указан</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>921709</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Трек В</t>
-        </is>
-      </c>
-      <c r="C10">
-        <v>39</v>
-      </c>
-      <c r="D10">
-        <v>79.032891</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>статус не указан</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>190122</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Трек А</t>
-        </is>
-      </c>
-      <c r="C11">
-        <v>41</v>
-      </c>
-      <c r="D11">
-        <v>77.704375</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>статус не указан</t>
-        </is>
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -1664,6 +1966,270 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>id ученика</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>трек</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>место в рейтинге</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>рейтинг</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>статус без выбора</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>637756</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Трек А</t>
+        </is>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2">
+        <v>100.004709</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>статус не указан</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>366609</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Трек В</t>
+        </is>
+      </c>
+      <c r="C3">
+        <v>5</v>
+      </c>
+      <c r="D3">
+        <v>100.004692</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>статус не указан</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>449867</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Трек А</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>9</v>
+      </c>
+      <c r="D4">
+        <v>99.492375</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>статус не указан</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>302756</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Трек А</t>
+        </is>
+      </c>
+      <c r="C5">
+        <v>13</v>
+      </c>
+      <c r="D5">
+        <v>97.987142</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>статус не указан</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>254592</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Трек А</t>
+        </is>
+      </c>
+      <c r="C6">
+        <v>17</v>
+      </c>
+      <c r="D6">
+        <v>96.805618</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>статус не указан</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>473699</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Трек С</t>
+        </is>
+      </c>
+      <c r="C7">
+        <v>22</v>
+      </c>
+      <c r="D7">
+        <v>95.028425</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>статус не указан</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>406855</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Трек А</t>
+        </is>
+      </c>
+      <c r="C8">
+        <v>34</v>
+      </c>
+      <c r="D8">
+        <v>87.061286</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>статус не указан</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>754466</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Трек В</t>
+        </is>
+      </c>
+      <c r="C9">
+        <v>37</v>
+      </c>
+      <c r="D9">
+        <v>83.014029</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>статус не указан</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>921709</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Трек В</t>
+        </is>
+      </c>
+      <c r="C10">
+        <v>39</v>
+      </c>
+      <c r="D10">
+        <v>79.032891</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>статус не указан</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>190122</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Трек А</t>
+        </is>
+      </c>
+      <c r="C11">
+        <v>41</v>
+      </c>
+      <c r="D11">
+        <v>77.704375</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>статус не указан</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
           <t>трек</t>
         </is>
       </c>

</xml_diff>